<commit_message>
Redesign chart as a per-asset Sankey-style cash flow diagram
Replace the line/area budget graph with a flow diagram: a central balance
trunk (thickness = balance) with one colored ribbon per asset that merges
in (IN, thickens the trunk) or peels off (OUT, thins it) at its
transaction date, connecting to a labeled pill above/below the trunk.
Ribbon/pill colors use the validated categorical palette from the dataviz
skill. Pills auto-stack to avoid overlap and clamp to the chart edges.
</commit_message>
<xml_diff>
--- a/InputExample.xlsx
+++ b/InputExample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janburianek/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janburianek/Projects/CashFlowViz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BFEE2E3-811A-C844-8737-BAD292083B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A17C4E2-DFA8-3A48-9E09-FEBFA172D3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20280" yWindow="5460" windowWidth="28240" windowHeight="17240" xr2:uid="{D6FAB51D-F143-6D4A-8384-8535D8013602}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Proj 1</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>STATUS</t>
+  </si>
+  <si>
+    <t>Hala nájem</t>
   </si>
 </sst>
 </file>
@@ -68,7 +71,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;Kč&quot;_-;\-* #,##0.00\ &quot;Kč&quot;_-;_-* &quot;-&quot;??\ &quot;Kč&quot;_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0\ &quot;Kč&quot;_-;\-* #,##0\ &quot;Kč&quot;_-;_-* &quot;-&quot;??\ &quot;Kč&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0\ &quot;Kč&quot;_-;\-* #,##0\ &quot;Kč&quot;_-;_-* &quot;-&quot;??\ &quot;Kč&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -119,7 +122,7 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -457,11 +460,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4904BBF0-813C-5A48-ABFD-FDD141CD3DAA}">
-  <dimension ref="B2:D6"/>
+  <dimension ref="B2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
@@ -519,6 +522,17 @@
         <v>-140000</v>
       </c>
     </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1">
+        <v>46266</v>
+      </c>
+      <c r="D7" s="2">
+        <v>-500000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace ribbon connectors with dotted leader lines to the trunk
Each transaction now connects to the graph with a thin dashed line (IN
pills draw straight down, OUT pills straight up) ending in a small dot at
the exact point on the balance trunk, instead of a filled Sankey ribbon.
</commit_message>
<xml_diff>
--- a/InputExample.xlsx
+++ b/InputExample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janburianek/Projects/CashFlowViz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A17C4E2-DFA8-3A48-9E09-FEBFA172D3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528DD99A-9116-3646-A1E3-2ED064F06737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20280" yWindow="5460" windowWidth="28240" windowHeight="17240" xr2:uid="{D6FAB51D-F143-6D4A-8384-8535D8013602}"/>
+    <workbookView xWindow="22020" yWindow="7680" windowWidth="28240" windowHeight="17240" xr2:uid="{D6FAB51D-F143-6D4A-8384-8535D8013602}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
   <si>
     <t>Proj 1</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Hala nájem</t>
+  </si>
+  <si>
+    <t>Neflix FR</t>
   </si>
 </sst>
 </file>
@@ -460,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4904BBF0-813C-5A48-ABFD-FDD141CD3DAA}">
-  <dimension ref="B2:D7"/>
+  <dimension ref="B2:D12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.6640625" customWidth="1"/>
@@ -524,12 +527,67 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1">
+        <v>46280</v>
+      </c>
+      <c r="D7" s="2">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C8" s="1">
         <v>46266</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D8" s="2">
+        <v>-500000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1">
+        <v>46296</v>
+      </c>
+      <c r="D9" s="2">
+        <v>-500000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1">
+        <v>46327</v>
+      </c>
+      <c r="D10" s="2">
+        <v>-500000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1">
+        <v>46357</v>
+      </c>
+      <c r="D11" s="2">
+        <v>-500000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1">
+        <v>46388</v>
+      </c>
+      <c r="D12" s="2">
         <v>-500000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add multi-column Sankey diagram tool (cashflowviz.sankey)
New, separate visualization on this branch: reads a FROM/AMOUNT/DATE
workbook and renders a literal Sankey diagram — income sources and
expense sinks as their own flexible columns, joined through gray
month-hub nodes that carry the running balance forward (turning red on
a deficit), in the style of the classic Microsoft "Cash Flow Template".

Column position is derived directly from the graph structure (income for
month m at column 2m-1, hub at 2m, expenses at 2m+1) rather than a
generic Sankey layout algorithm, since the shape is fully known upfront.

Independent of the existing cashflowviz package/CLI, which is unchanged.
</commit_message>
<xml_diff>
--- a/InputExample.xlsx
+++ b/InputExample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janburianek/Projects/CashFlowViz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528DD99A-9116-3646-A1E3-2ED064F06737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89F7EA9D-A4C3-9B4C-B1AF-FC935E17B505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22020" yWindow="7680" windowWidth="28240" windowHeight="17240" xr2:uid="{D6FAB51D-F143-6D4A-8384-8535D8013602}"/>
   </bookViews>
@@ -59,13 +59,13 @@
     <t>Jan B</t>
   </si>
   <si>
-    <t>STATUS</t>
-  </si>
-  <si>
     <t>Hala nájem</t>
   </si>
   <si>
     <t>Neflix FR</t>
+  </si>
+  <si>
+    <t>START</t>
   </si>
 </sst>
 </file>
@@ -483,7 +483,7 @@
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1">
         <v>46251</v>
@@ -527,7 +527,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="1">
         <v>46280</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1">
         <v>46266</v>
@@ -549,7 +549,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" s="1">
         <v>46296</v>
@@ -560,7 +560,7 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" s="1">
         <v>46327</v>
@@ -571,7 +571,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1">
         <v>46357</v>
@@ -582,7 +582,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" s="1">
         <v>46388</v>

</xml_diff>

<commit_message>
Unify both tools onto one FROM/AMOUNT/DATE input format
Both cashflowviz and cashflowviz.sankey now read the exact same workbook
shape and parser (new cashflowviz/io.py, extracted from what was
cashflowviz.sankey's reader). They still produce different diagrams, but
the same .xlsx now works with either --  the balance-trunk and the
Sankey renderer are purely two views over the same data.

This drops the old Assets/Date/IN-OUT layout and its magic STATUS row:
an opening balance is now just a normal positive-amount entry (as it
already was in the Sankey tool), with the running balance starting at 0
for both tools. In the trunk diagram, that means the opening entry now
gets its own pill and dashed connector like any other transaction,
ramping the trunk up from 0, rather than starting flat.

InputExample.xlsx's headers are renamed to FROM/AMOUNT/DATE to match;
its data is unchanged, and it now works with cashflowviz.sankey too.
</commit_message>
<xml_diff>
--- a/InputExample.xlsx
+++ b/InputExample.xlsx
@@ -1,109 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janburianek/Projects/CashFlowViz/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89F7EA9D-A4C3-9B4C-B1AF-FC935E17B505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="22020" yWindow="7680" windowWidth="28240" windowHeight="17240" xr2:uid="{D6FAB51D-F143-6D4A-8384-8535D8013602}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="22020" yWindow="7680" windowWidth="28240" windowHeight="17240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="List1" sheetId="1" r:id="rId1"/>
+    <sheet name="List1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
-  <si>
-    <t>Proj 1</t>
-  </si>
-  <si>
-    <t>Assets</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>IN/OUT</t>
-  </si>
-  <si>
-    <t>Tomáš N</t>
-  </si>
-  <si>
-    <t>Jan B</t>
-  </si>
-  <si>
-    <t>Hala nájem</t>
-  </si>
-  <si>
-    <t>Neflix FR</t>
-  </si>
-  <si>
-    <t>START</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;Kč&quot;_-;\-* #,##0.00\ &quot;Kč&quot;_-;_-* &quot;-&quot;??\ &quot;Kč&quot;_-;_-@_-"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0\ &quot;Kč&quot;_-;\-* #,##0\ &quot;Kč&quot;_-;_-* &quot;-&quot;??\ &quot;Kč&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -119,30 +61,89 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normální" xfId="0" builtinId="0"/>
     <cellStyle name="Měna" xfId="1" builtinId="4"/>
-    <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -462,136 +463,166 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4904BBF0-813C-5A48-ABFD-FDD141CD3DAA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col width="6.6640625" customWidth="1" min="1" max="1"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1">
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>FROM</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>AMOUNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
         <v>46251</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="2" t="n">
         <v>1000000</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1">
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Proj 1</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
         <v>46254</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="2" t="n">
         <v>100000</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="1">
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tomáš N</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
         <v>46260</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="2" t="n">
         <v>-100000</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1">
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jan B</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>46273</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="2" t="n">
         <v>-140000</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="1">
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Neflix FR</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="2" t="n">
         <v>800000</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1">
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hala nájem</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="2" t="n">
         <v>-500000</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="1">
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hala nájem</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
         <v>46296</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="2" t="n">
         <v>-500000</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="1">
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hala nájem</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="2" t="n">
         <v>-500000</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="1">
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Hala nájem</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>46357</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="2" t="n">
         <v>-500000</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="1">
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hala nájem</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="n">
         <v>46388</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="2" t="n">
         <v>-500000</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>